<commit_message>
AML1 analysis for plants
</commit_message>
<xml_diff>
--- a/datasets/Pflanzenauswertung-Template_new.xlsx
+++ b/datasets/Pflanzenauswertung-Template_new.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wageningenur4-my.sharepoint.com/personal/luciana_chavezrodriguez_wur_nl/Documents/UCI_projects/Project_8 (Reviews)/Family/Pere/doctorado/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucia\OneDrive - Wageningen University &amp; Research\UCI_projects\Project_8 (Reviews)\Family\Pere\doctorado\datasets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="168" documentId="11_9E4C551FCCD8CC5256BC57F0ABB953959291F851" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D9C0DBD7-5C05-4C93-8793-3535614591CD}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E6DAE14-AD91-4714-BBEB-840F5992E8A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle 1" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="530" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="569" uniqueCount="68">
   <si>
     <t>spore conc. 1x10^7 Sp/ml, infection 40 min root dipping while shaking (35 rpm)</t>
   </si>
@@ -265,6 +265,15 @@
   </si>
   <si>
     <t xml:space="preserve">oeLLM1 </t>
+  </si>
+  <si>
+    <t>treatments</t>
+  </si>
+  <si>
+    <t>Percent</t>
+  </si>
+  <si>
+    <t>rank</t>
   </si>
 </sst>
 </file>
@@ -7826,6 +7835,50 @@
   </sheetData>
   <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
   <mergeCells count="52">
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="D7:D8"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="I9:I10"/>
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="K9:K10"/>
+    <mergeCell ref="B43:B44"/>
+    <mergeCell ref="C43:C44"/>
+    <mergeCell ref="D43:D44"/>
+    <mergeCell ref="E43:E44"/>
+    <mergeCell ref="H9:H10"/>
+    <mergeCell ref="B64:B65"/>
+    <mergeCell ref="C64:C65"/>
+    <mergeCell ref="D64:D65"/>
+    <mergeCell ref="E64:E65"/>
+    <mergeCell ref="B85:B86"/>
+    <mergeCell ref="C85:C86"/>
+    <mergeCell ref="D85:D86"/>
+    <mergeCell ref="E85:E86"/>
+    <mergeCell ref="B106:B107"/>
+    <mergeCell ref="C106:C107"/>
+    <mergeCell ref="D106:D107"/>
+    <mergeCell ref="E106:E107"/>
+    <mergeCell ref="B127:B128"/>
+    <mergeCell ref="C127:C128"/>
+    <mergeCell ref="D127:D128"/>
+    <mergeCell ref="E127:E128"/>
+    <mergeCell ref="B148:B149"/>
+    <mergeCell ref="C148:C149"/>
+    <mergeCell ref="D148:D149"/>
+    <mergeCell ref="E148:E149"/>
+    <mergeCell ref="B169:B170"/>
+    <mergeCell ref="C169:C170"/>
+    <mergeCell ref="D169:D170"/>
+    <mergeCell ref="E169:E170"/>
+    <mergeCell ref="B190:B191"/>
+    <mergeCell ref="C190:C191"/>
+    <mergeCell ref="D190:D191"/>
+    <mergeCell ref="E190:E191"/>
+    <mergeCell ref="B211:B212"/>
+    <mergeCell ref="C211:C212"/>
+    <mergeCell ref="D211:D212"/>
+    <mergeCell ref="E211:E212"/>
     <mergeCell ref="B232:B233"/>
     <mergeCell ref="C232:C233"/>
     <mergeCell ref="D232:D233"/>
@@ -7834,50 +7887,6 @@
     <mergeCell ref="C253:C254"/>
     <mergeCell ref="D253:D254"/>
     <mergeCell ref="E253:E254"/>
-    <mergeCell ref="B190:B191"/>
-    <mergeCell ref="C190:C191"/>
-    <mergeCell ref="D190:D191"/>
-    <mergeCell ref="E190:E191"/>
-    <mergeCell ref="B211:B212"/>
-    <mergeCell ref="C211:C212"/>
-    <mergeCell ref="D211:D212"/>
-    <mergeCell ref="E211:E212"/>
-    <mergeCell ref="B148:B149"/>
-    <mergeCell ref="C148:C149"/>
-    <mergeCell ref="D148:D149"/>
-    <mergeCell ref="E148:E149"/>
-    <mergeCell ref="B169:B170"/>
-    <mergeCell ref="C169:C170"/>
-    <mergeCell ref="D169:D170"/>
-    <mergeCell ref="E169:E170"/>
-    <mergeCell ref="B106:B107"/>
-    <mergeCell ref="C106:C107"/>
-    <mergeCell ref="D106:D107"/>
-    <mergeCell ref="E106:E107"/>
-    <mergeCell ref="B127:B128"/>
-    <mergeCell ref="C127:C128"/>
-    <mergeCell ref="D127:D128"/>
-    <mergeCell ref="E127:E128"/>
-    <mergeCell ref="B64:B65"/>
-    <mergeCell ref="C64:C65"/>
-    <mergeCell ref="D64:D65"/>
-    <mergeCell ref="E64:E65"/>
-    <mergeCell ref="B85:B86"/>
-    <mergeCell ref="C85:C86"/>
-    <mergeCell ref="D85:D86"/>
-    <mergeCell ref="E85:E86"/>
-    <mergeCell ref="J9:J10"/>
-    <mergeCell ref="K9:K10"/>
-    <mergeCell ref="B43:B44"/>
-    <mergeCell ref="C43:C44"/>
-    <mergeCell ref="D43:D44"/>
-    <mergeCell ref="E43:E44"/>
-    <mergeCell ref="H9:H10"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="D7:D8"/>
-    <mergeCell ref="E7:E8"/>
-    <mergeCell ref="I9:I10"/>
   </mergeCells>
   <pageMargins left="0.70833333333333337" right="0.70833333333333337" top="0.78749999999999998" bottom="0.78749999999999998" header="0.51180555555555551" footer="0.51180555555555551"/>
   <pageSetup paperSize="9" scale="45" firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -9232,7 +9241,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:R269"/>
+  <dimension ref="A1:Z269"/>
   <sheetFormatPr defaultColWidth="10.88671875" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="11" width="10.88671875" style="1"/>
@@ -9241,10 +9250,12 @@
     <col min="15" max="15" width="10.88671875" style="1" customWidth="1"/>
     <col min="16" max="16" width="14.21875" style="1" customWidth="1"/>
     <col min="17" max="17" width="14.109375" style="1" customWidth="1"/>
-    <col min="18" max="16384" width="10.88671875" style="1"/>
+    <col min="18" max="19" width="10.88671875" style="1"/>
+    <col min="20" max="20" width="20.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="21" max="16384" width="10.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A1" s="19" t="str">
         <f>'Tabelle 1'!A7</f>
         <v>Mock A</v>
@@ -9285,8 +9296,29 @@
       <c r="R1" s="35" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="U1" s="35" t="s">
+        <v>58</v>
+      </c>
+      <c r="V1" s="35" t="s">
+        <v>56</v>
+      </c>
+      <c r="W1" s="35" t="s">
+        <v>60</v>
+      </c>
+      <c r="X1" s="35" t="s">
+        <v>62</v>
+      </c>
+      <c r="Y1" s="36" t="s">
+        <v>63</v>
+      </c>
+      <c r="Z1" s="35" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A2" s="12">
         <v>1</v>
       </c>
@@ -9343,8 +9375,35 @@
         <f>SUM(O12+O19+O26+O33)</f>
         <v>59</v>
       </c>
-    </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T2" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="U2" s="1">
+        <f>M2/M$8</f>
+        <v>0.98333333333333328</v>
+      </c>
+      <c r="V2" s="1">
+        <f>N2/N$8</f>
+        <v>0.17222222222222222</v>
+      </c>
+      <c r="W2" s="1">
+        <f>O2/O$8</f>
+        <v>0.39333333333333331</v>
+      </c>
+      <c r="X2" s="1">
+        <f>P2/P$8</f>
+        <v>0.18333333333333332</v>
+      </c>
+      <c r="Y2" s="1">
+        <f>Q2/Q$8</f>
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="Z2" s="1">
+        <f>R2/R$8</f>
+        <v>0.32777777777777778</v>
+      </c>
+    </row>
+    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A3" s="12">
         <v>2</v>
       </c>
@@ -9400,8 +9459,35 @@
         <f>SUM(O13+O20+O27+O34)</f>
         <v>68</v>
       </c>
-    </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T3" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="U3" s="1">
+        <f t="shared" ref="U3:U8" si="1">M3/M$8</f>
+        <v>1.6666666666666666E-2</v>
+      </c>
+      <c r="V3" s="1">
+        <f t="shared" ref="V3:V6" si="2">N3/N$8</f>
+        <v>0.36666666666666664</v>
+      </c>
+      <c r="W3" s="1">
+        <f t="shared" ref="W3:W6" si="3">O3/O$8</f>
+        <v>0.36</v>
+      </c>
+      <c r="X3" s="1">
+        <f t="shared" ref="X3:X6" si="4">P3/P$8</f>
+        <v>0.23333333333333334</v>
+      </c>
+      <c r="Y3" s="1">
+        <f t="shared" ref="Y3:Y6" si="5">Q3/Q$8</f>
+        <v>0.23333333333333334</v>
+      </c>
+      <c r="Z3" s="1">
+        <f t="shared" ref="Z3:Z6" si="6">R3/R$8</f>
+        <v>0.37777777777777777</v>
+      </c>
+    </row>
+    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A4" s="12">
         <v>3</v>
       </c>
@@ -9458,8 +9544,35 @@
         <f>SUM(O14+O21+O28+O35)</f>
         <v>44</v>
       </c>
-    </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T4" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="U4" s="1">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="V4" s="1">
+        <f t="shared" si="2"/>
+        <v>0.3611111111111111</v>
+      </c>
+      <c r="W4" s="1">
+        <f t="shared" si="3"/>
+        <v>0.21333333333333335</v>
+      </c>
+      <c r="X4" s="1">
+        <f t="shared" si="4"/>
+        <v>0.53333333333333333</v>
+      </c>
+      <c r="Y4" s="1">
+        <f t="shared" si="5"/>
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="Z4" s="1">
+        <f t="shared" si="6"/>
+        <v>0.24444444444444444</v>
+      </c>
+    </row>
+    <row r="5" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A5" s="12">
         <v>4</v>
       </c>
@@ -9515,8 +9628,35 @@
         <f>SUM(O15+O22+O29+O36)</f>
         <v>9</v>
       </c>
-    </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T5" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="U5" s="1">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="V5" s="1">
+        <f t="shared" si="2"/>
+        <v>0.1</v>
+      </c>
+      <c r="W5" s="1">
+        <f t="shared" si="3"/>
+        <v>3.3333333333333333E-2</v>
+      </c>
+      <c r="X5" s="1">
+        <f t="shared" si="4"/>
+        <v>0.05</v>
+      </c>
+      <c r="Y5" s="1">
+        <f t="shared" si="5"/>
+        <v>0.1</v>
+      </c>
+      <c r="Z5" s="1">
+        <f t="shared" si="6"/>
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A6" s="12">
         <v>5</v>
       </c>
@@ -9571,8 +9711,35 @@
       <c r="R6" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T6" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="U6" s="1">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="V6" s="1">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="W6" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="X6" s="1">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Y6" s="1">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="Z6" s="1">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A7" s="12">
         <v>6</v>
       </c>
@@ -9597,7 +9764,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A8" s="12">
         <v>7</v>
       </c>
@@ -9625,27 +9792,27 @@
         <v>180</v>
       </c>
       <c r="N8" s="1">
-        <f t="shared" ref="N8:R8" si="1">SUM(N2:N6)</f>
+        <f t="shared" ref="N8:R8" si="7">SUM(N2:N6)</f>
         <v>180</v>
       </c>
       <c r="O8" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="7"/>
         <v>150</v>
       </c>
       <c r="P8" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="7"/>
         <v>60</v>
       </c>
       <c r="Q8" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="7"/>
         <v>30</v>
       </c>
       <c r="R8" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="7"/>
         <v>180</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A9" s="12">
         <v>8</v>
       </c>
@@ -9666,7 +9833,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A10" s="12">
         <v>9</v>
       </c>
@@ -9686,8 +9853,17 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-    </row>
-    <row r="11" spans="1:18" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="U10" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="V10" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="W10" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="11" spans="1:26" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A11" s="12">
         <v>10</v>
       </c>
@@ -9719,8 +9895,17 @@
       <c r="P11" s="1" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="U11" s="35" t="s">
+        <v>58</v>
+      </c>
+      <c r="V11" s="1">
+        <v>0.98333333333333328</v>
+      </c>
+      <c r="W11" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A12" s="12">
         <v>11</v>
       </c>
@@ -9752,8 +9937,17 @@
       <c r="P12" s="1">
         <v>34</v>
       </c>
-    </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="U12" s="35" t="s">
+        <v>58</v>
+      </c>
+      <c r="V12" s="1">
+        <v>1.6666666666666666E-2</v>
+      </c>
+      <c r="W12" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A13" s="12">
         <v>12</v>
       </c>
@@ -9785,8 +9979,17 @@
       <c r="P13" s="1">
         <v>26</v>
       </c>
-    </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="U13" s="35" t="s">
+        <v>58</v>
+      </c>
+      <c r="V13" s="1">
+        <v>0</v>
+      </c>
+      <c r="W13" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A14" s="12">
         <v>13</v>
       </c>
@@ -9820,8 +10023,17 @@
         <f>H182</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="U14" s="35" t="s">
+        <v>58</v>
+      </c>
+      <c r="V14" s="1">
+        <v>0</v>
+      </c>
+      <c r="W14" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A15" s="12">
         <v>14</v>
       </c>
@@ -9857,8 +10069,17 @@
         <f>H183</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="U15" s="35" t="s">
+        <v>56</v>
+      </c>
+      <c r="V15" s="1">
+        <v>0.17222222222222222</v>
+      </c>
+      <c r="W15" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A16" s="12">
         <v>15</v>
       </c>
@@ -9894,8 +10115,17 @@
         <f>H184</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="U16" s="35" t="s">
+        <v>56</v>
+      </c>
+      <c r="V16" s="1">
+        <v>0.36666666666666664</v>
+      </c>
+      <c r="W16" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A17" s="12"/>
       <c r="B17" s="12"/>
       <c r="C17" s="12"/>
@@ -9904,8 +10134,17 @@
       <c r="F17" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="U17" s="35" t="s">
+        <v>56</v>
+      </c>
+      <c r="V17" s="1">
+        <v>0.3611111111111111</v>
+      </c>
+      <c r="W17" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A18" s="19" t="s">
         <v>48</v>
       </c>
@@ -9938,8 +10177,17 @@
       <c r="O18" s="1" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="U18" s="35" t="s">
+        <v>56</v>
+      </c>
+      <c r="V18" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="W18" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A19" s="19" t="s">
         <v>49</v>
       </c>
@@ -9968,8 +10216,17 @@
       <c r="O19" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="U19" s="35" t="s">
+        <v>60</v>
+      </c>
+      <c r="V19" s="1">
+        <v>0.39333333333333331</v>
+      </c>
+      <c r="W19" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:23" x14ac:dyDescent="0.25">
       <c r="M20" s="1">
         <v>1</v>
       </c>
@@ -9979,8 +10236,17 @@
       <c r="O20" s="1">
         <v>16</v>
       </c>
-    </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="U20" s="35" t="s">
+        <v>60</v>
+      </c>
+      <c r="V20" s="1">
+        <v>0.36</v>
+      </c>
+      <c r="W20" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:23" x14ac:dyDescent="0.25">
       <c r="M21" s="1">
         <v>0</v>
       </c>
@@ -9990,8 +10256,17 @@
       <c r="O21" s="1">
         <v>11</v>
       </c>
-    </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="U21" s="35" t="s">
+        <v>60</v>
+      </c>
+      <c r="V21" s="1">
+        <v>0.21333333333333335</v>
+      </c>
+      <c r="W21" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A22" s="19" t="str">
         <f>'Tabelle 1'!A43</f>
         <v>Mock B</v>
@@ -10020,8 +10295,17 @@
       <c r="O22" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="U22" s="35" t="s">
+        <v>60</v>
+      </c>
+      <c r="V22" s="1">
+        <v>3.3333333333333333E-2</v>
+      </c>
+      <c r="W22" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A23" s="12">
         <v>1</v>
       </c>
@@ -10038,7 +10322,7 @@
         <v>5</v>
       </c>
       <c r="E23" s="17">
-        <f t="shared" ref="E23:E37" si="2">AVERAGE(B23:D23)</f>
+        <f t="shared" ref="E23:E37" si="8">AVERAGE(B23:D23)</f>
         <v>5</v>
       </c>
       <c r="G23" s="34" t="s">
@@ -10057,8 +10341,17 @@
       <c r="O23" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="U23" s="35" t="s">
+        <v>62</v>
+      </c>
+      <c r="V23" s="1">
+        <v>0.18333333333333332</v>
+      </c>
+      <c r="W23" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A24" s="12">
         <v>2</v>
       </c>
@@ -10075,7 +10368,7 @@
         <v>5</v>
       </c>
       <c r="E24" s="17">
-        <f t="shared" si="2"/>
+        <f t="shared" si="8"/>
         <v>5</v>
       </c>
       <c r="G24" s="34" t="s">
@@ -10085,8 +10378,17 @@
         <f>COUNTIFS($E$23:$E$37,"&lt;2,99",$E$23:$E$37,"&gt;=2")</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="U24" s="35" t="s">
+        <v>62</v>
+      </c>
+      <c r="V24" s="1">
+        <v>0.23333333333333334</v>
+      </c>
+      <c r="W24" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A25" s="12">
         <v>3</v>
       </c>
@@ -10103,7 +10405,7 @@
         <v>5</v>
       </c>
       <c r="E25" s="17">
-        <f t="shared" si="2"/>
+        <f t="shared" si="8"/>
         <v>5</v>
       </c>
       <c r="G25" s="34" t="s">
@@ -10122,8 +10424,17 @@
       <c r="O25" s="1" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="U25" s="35" t="s">
+        <v>62</v>
+      </c>
+      <c r="V25" s="1">
+        <v>0.53333333333333333</v>
+      </c>
+      <c r="W25" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A26" s="12">
         <v>4</v>
       </c>
@@ -10140,7 +10451,7 @@
         <v>5</v>
       </c>
       <c r="E26" s="17">
-        <f t="shared" si="2"/>
+        <f t="shared" si="8"/>
         <v>5</v>
       </c>
       <c r="G26" s="34" t="s">
@@ -10159,8 +10470,17 @@
       <c r="O26" s="1">
         <v>20</v>
       </c>
-    </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="U26" s="35" t="s">
+        <v>62</v>
+      </c>
+      <c r="V26" s="1">
+        <v>0.05</v>
+      </c>
+      <c r="W26" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="27" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A27" s="12">
         <v>5</v>
       </c>
@@ -10177,7 +10497,7 @@
         <v>5</v>
       </c>
       <c r="E27" s="17">
-        <f t="shared" si="2"/>
+        <f t="shared" si="8"/>
         <v>5</v>
       </c>
       <c r="G27" s="34">
@@ -10196,8 +10516,17 @@
       <c r="O27" s="1">
         <v>8</v>
       </c>
-    </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="U27" s="36" t="s">
+        <v>63</v>
+      </c>
+      <c r="V27" s="1">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="W27" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A28" s="12">
         <v>6</v>
       </c>
@@ -10214,7 +10543,7 @@
         <v>5</v>
       </c>
       <c r="E28" s="17">
-        <f t="shared" si="2"/>
+        <f t="shared" si="8"/>
         <v>5</v>
       </c>
       <c r="H28" s="1">
@@ -10230,8 +10559,17 @@
       <c r="O28" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="U28" s="36" t="s">
+        <v>63</v>
+      </c>
+      <c r="V28" s="1">
+        <v>0.23333333333333334</v>
+      </c>
+      <c r="W28" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A29" s="12">
         <v>7</v>
       </c>
@@ -10248,7 +10586,7 @@
         <v>5</v>
       </c>
       <c r="E29" s="17">
-        <f t="shared" si="2"/>
+        <f t="shared" si="8"/>
         <v>5</v>
       </c>
       <c r="M29" s="1">
@@ -10260,8 +10598,17 @@
       <c r="O29" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="U29" s="36" t="s">
+        <v>63</v>
+      </c>
+      <c r="V29" s="1">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="W29" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A30" s="12">
         <v>8</v>
       </c>
@@ -10278,7 +10625,7 @@
         <v>5</v>
       </c>
       <c r="E30" s="17">
-        <f t="shared" si="2"/>
+        <f t="shared" si="8"/>
         <v>5</v>
       </c>
       <c r="F30" s="1" t="s">
@@ -10293,8 +10640,17 @@
       <c r="O30" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="U30" s="36" t="s">
+        <v>63</v>
+      </c>
+      <c r="V30" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="W30" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="31" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A31" s="12">
         <v>9</v>
       </c>
@@ -10311,14 +10667,23 @@
         <v>5</v>
       </c>
       <c r="E31" s="17">
-        <f t="shared" si="2"/>
+        <f t="shared" si="8"/>
         <v>5</v>
       </c>
       <c r="G31" s="33"/>
       <c r="H31" s="33"/>
       <c r="I31" s="33"/>
-    </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="U31" s="35" t="s">
+        <v>59</v>
+      </c>
+      <c r="V31" s="1">
+        <v>0.32777777777777778</v>
+      </c>
+      <c r="W31" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A32" s="12">
         <v>10</v>
       </c>
@@ -10335,7 +10700,7 @@
         <v>5</v>
       </c>
       <c r="E32" s="17">
-        <f t="shared" si="2"/>
+        <f t="shared" si="8"/>
         <v>5</v>
       </c>
       <c r="G32" s="33"/>
@@ -10350,8 +10715,17 @@
       <c r="O32" s="1" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="33" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="U32" s="35" t="s">
+        <v>59</v>
+      </c>
+      <c r="V32" s="1">
+        <v>0.37777777777777777</v>
+      </c>
+      <c r="W32" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="33" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A33" s="12">
         <v>11</v>
       </c>
@@ -10368,7 +10742,7 @@
         <v>5</v>
       </c>
       <c r="E33" s="17">
-        <f t="shared" si="2"/>
+        <f t="shared" si="8"/>
         <v>5</v>
       </c>
       <c r="G33" s="33"/>
@@ -10383,8 +10757,17 @@
       <c r="O33" s="1">
         <v>9</v>
       </c>
-    </row>
-    <row r="34" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="U33" s="35" t="s">
+        <v>59</v>
+      </c>
+      <c r="V33" s="1">
+        <v>0.24444444444444444</v>
+      </c>
+      <c r="W33" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A34" s="12">
         <v>12</v>
       </c>
@@ -10401,7 +10784,7 @@
         <v>5</v>
       </c>
       <c r="E34" s="17">
-        <f t="shared" si="2"/>
+        <f t="shared" si="8"/>
         <v>5</v>
       </c>
       <c r="G34" s="33"/>
@@ -10416,8 +10799,17 @@
       <c r="O34" s="1">
         <v>21</v>
       </c>
-    </row>
-    <row r="35" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="U34" s="35" t="s">
+        <v>59</v>
+      </c>
+      <c r="V34" s="1">
+        <v>0.05</v>
+      </c>
+      <c r="W34" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="35" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A35" s="12">
         <v>13</v>
       </c>
@@ -10434,7 +10826,7 @@
         <v>5</v>
       </c>
       <c r="E35" s="17">
-        <f t="shared" si="2"/>
+        <f t="shared" si="8"/>
         <v>5</v>
       </c>
       <c r="G35" s="33"/>
@@ -10450,7 +10842,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="36" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A36" s="12">
         <v>14</v>
       </c>
@@ -10467,7 +10859,7 @@
         <v>5</v>
       </c>
       <c r="E36" s="17">
-        <f t="shared" si="2"/>
+        <f t="shared" si="8"/>
         <v>5</v>
       </c>
       <c r="G36" s="33"/>
@@ -10483,7 +10875,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="37" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A37" s="12">
         <v>15</v>
       </c>
@@ -10500,7 +10892,7 @@
         <v>5</v>
       </c>
       <c r="E37" s="17">
-        <f t="shared" si="2"/>
+        <f t="shared" si="8"/>
         <v>5</v>
       </c>
       <c r="M37" s="1">
@@ -10513,7 +10905,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A38" s="12"/>
       <c r="B38" s="12"/>
       <c r="C38" s="12"/>
@@ -10523,7 +10915,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="39" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A39" s="19" t="s">
         <v>48</v>
       </c>
@@ -10563,7 +10955,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="40" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A40" s="19" t="s">
         <v>49</v>
       </c>
@@ -10599,7 +10991,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="41" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:23" x14ac:dyDescent="0.25">
       <c r="M41" s="1">
         <v>0</v>
       </c>
@@ -10616,7 +11008,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="42" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:23" x14ac:dyDescent="0.25">
       <c r="M42" s="1">
         <v>0</v>
       </c>
@@ -10633,7 +11025,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="43" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A43" s="9">
         <f>'Tabelle 1'!A64</f>
         <v>3</v>
@@ -10669,7 +11061,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="44" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A44" s="12">
         <v>1</v>
       </c>
@@ -10686,7 +11078,7 @@
         <v>5</v>
       </c>
       <c r="E44" s="17">
-        <f t="shared" ref="E44:E58" si="3">AVERAGE(B44:D44)</f>
+        <f t="shared" ref="E44:E58" si="9">AVERAGE(B44:D44)</f>
         <v>5</v>
       </c>
       <c r="G44" s="34" t="s">
@@ -10712,7 +11104,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A45" s="12">
         <v>2</v>
       </c>
@@ -10729,7 +11121,7 @@
         <v>5</v>
       </c>
       <c r="E45" s="17">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>5</v>
       </c>
       <c r="G45" s="34" t="s">
@@ -10740,7 +11132,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A46" s="12">
         <v>3</v>
       </c>
@@ -10757,7 +11149,7 @@
         <v>5</v>
       </c>
       <c r="E46" s="17">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>5</v>
       </c>
       <c r="G46" s="34" t="s">
@@ -10780,7 +11172,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="47" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A47" s="12">
         <v>4</v>
       </c>
@@ -10797,7 +11189,7 @@
         <v>5</v>
       </c>
       <c r="E47" s="17">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>5</v>
       </c>
       <c r="G47" s="34" t="s">
@@ -10820,7 +11212,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="48" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A48" s="12">
         <v>5</v>
       </c>
@@ -10837,7 +11229,7 @@
         <v>5</v>
       </c>
       <c r="E48" s="17">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>5</v>
       </c>
       <c r="G48" s="34">
@@ -10877,7 +11269,7 @@
         <v>5</v>
       </c>
       <c r="E49" s="17">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>5</v>
       </c>
       <c r="H49" s="1">
@@ -10914,7 +11306,7 @@
         <v>5</v>
       </c>
       <c r="E50" s="17">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>5</v>
       </c>
       <c r="M50" s="1">
@@ -10947,7 +11339,7 @@
         <v>5</v>
       </c>
       <c r="E51" s="17">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>5</v>
       </c>
       <c r="M51" s="1">
@@ -10980,7 +11372,7 @@
         <v>5</v>
       </c>
       <c r="E52" s="17">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>5</v>
       </c>
       <c r="G52" s="33"/>
@@ -11004,7 +11396,7 @@
         <v>5</v>
       </c>
       <c r="E53" s="17">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>5</v>
       </c>
       <c r="G53" s="33"/>
@@ -11028,7 +11420,7 @@
         <v>5</v>
       </c>
       <c r="E54" s="17">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>5</v>
       </c>
       <c r="G54" s="33"/>
@@ -11052,7 +11444,7 @@
         <v>5</v>
       </c>
       <c r="E55" s="17">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>5</v>
       </c>
       <c r="G55" s="33"/>
@@ -11076,7 +11468,7 @@
         <v>5</v>
       </c>
       <c r="E56" s="17">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>5</v>
       </c>
       <c r="G56" s="33"/>
@@ -11100,7 +11492,7 @@
         <v>5</v>
       </c>
       <c r="E57" s="17">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>5</v>
       </c>
       <c r="G57" s="33"/>
@@ -11124,7 +11516,7 @@
         <v>5</v>
       </c>
       <c r="E58" s="17">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>5</v>
       </c>
     </row>
@@ -11222,7 +11614,7 @@
         <v>5</v>
       </c>
       <c r="E65" s="17">
-        <f t="shared" ref="E65:E79" si="4">AVERAGE(B65:D65)</f>
+        <f t="shared" ref="E65:E79" si="10">AVERAGE(B65:D65)</f>
         <v>5</v>
       </c>
       <c r="G65" s="34" t="s">
@@ -11250,7 +11642,7 @@
         <v>5</v>
       </c>
       <c r="E66" s="17">
-        <f t="shared" si="4"/>
+        <f t="shared" si="10"/>
         <v>5</v>
       </c>
       <c r="G66" s="34" t="s">
@@ -11278,7 +11670,7 @@
         <v>5</v>
       </c>
       <c r="E67" s="17">
-        <f t="shared" si="4"/>
+        <f t="shared" si="10"/>
         <v>5</v>
       </c>
       <c r="G67" s="34" t="s">
@@ -11306,7 +11698,7 @@
         <v>5</v>
       </c>
       <c r="E68" s="17">
-        <f t="shared" si="4"/>
+        <f t="shared" si="10"/>
         <v>5</v>
       </c>
       <c r="G68" s="34" t="s">
@@ -11334,7 +11726,7 @@
         <v>5</v>
       </c>
       <c r="E69" s="17">
-        <f t="shared" si="4"/>
+        <f t="shared" si="10"/>
         <v>5</v>
       </c>
       <c r="G69" s="34">
@@ -11362,7 +11754,7 @@
         <v>5</v>
       </c>
       <c r="E70" s="17">
-        <f t="shared" si="4"/>
+        <f t="shared" si="10"/>
         <v>5</v>
       </c>
       <c r="H70" s="1">
@@ -11387,7 +11779,7 @@
         <v>5</v>
       </c>
       <c r="E71" s="17">
-        <f t="shared" si="4"/>
+        <f t="shared" si="10"/>
         <v>5</v>
       </c>
     </row>
@@ -11408,7 +11800,7 @@
         <v>5</v>
       </c>
       <c r="E72" s="17">
-        <f t="shared" si="4"/>
+        <f t="shared" si="10"/>
         <v>5</v>
       </c>
     </row>
@@ -11429,7 +11821,7 @@
         <v>5</v>
       </c>
       <c r="E73" s="17">
-        <f t="shared" si="4"/>
+        <f t="shared" si="10"/>
         <v>5</v>
       </c>
       <c r="G73" s="33"/>
@@ -11453,7 +11845,7 @@
         <v>5</v>
       </c>
       <c r="E74" s="17">
-        <f t="shared" si="4"/>
+        <f t="shared" si="10"/>
         <v>5</v>
       </c>
       <c r="G74" s="33"/>
@@ -11477,7 +11869,7 @@
         <v>5</v>
       </c>
       <c r="E75" s="17">
-        <f t="shared" si="4"/>
+        <f t="shared" si="10"/>
         <v>5</v>
       </c>
       <c r="G75" s="33"/>
@@ -11501,7 +11893,7 @@
         <v>5</v>
       </c>
       <c r="E76" s="17">
-        <f t="shared" si="4"/>
+        <f t="shared" si="10"/>
         <v>5</v>
       </c>
       <c r="G76" s="33"/>
@@ -11525,7 +11917,7 @@
         <v>5</v>
       </c>
       <c r="E77" s="17">
-        <f t="shared" si="4"/>
+        <f t="shared" si="10"/>
         <v>5</v>
       </c>
       <c r="G77" s="33"/>
@@ -11549,7 +11941,7 @@
         <v>5</v>
       </c>
       <c r="E78" s="17">
-        <f t="shared" si="4"/>
+        <f t="shared" si="10"/>
         <v>5</v>
       </c>
       <c r="G78" s="33"/>
@@ -11573,7 +11965,7 @@
         <v>5</v>
       </c>
       <c r="E79" s="17">
-        <f t="shared" si="4"/>
+        <f t="shared" si="10"/>
         <v>5</v>
       </c>
     </row>
@@ -11671,7 +12063,7 @@
         <v>5</v>
       </c>
       <c r="E86" s="17">
-        <f t="shared" ref="E86:E100" si="5">AVERAGE(B86:D86)</f>
+        <f t="shared" ref="E86:E100" si="11">AVERAGE(B86:D86)</f>
         <v>5</v>
       </c>
       <c r="G86" s="34" t="s">
@@ -11699,7 +12091,7 @@
         <v>5</v>
       </c>
       <c r="E87" s="17">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>5</v>
       </c>
       <c r="G87" s="34" t="s">
@@ -11727,7 +12119,7 @@
         <v>5</v>
       </c>
       <c r="E88" s="17">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>5</v>
       </c>
       <c r="G88" s="34" t="s">
@@ -11755,7 +12147,7 @@
         <v>5</v>
       </c>
       <c r="E89" s="17">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>5</v>
       </c>
       <c r="G89" s="34" t="s">
@@ -11783,7 +12175,7 @@
         <v>5</v>
       </c>
       <c r="E90" s="17">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>5</v>
       </c>
       <c r="G90" s="34">
@@ -11811,7 +12203,7 @@
         <v>5</v>
       </c>
       <c r="E91" s="17">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>5</v>
       </c>
       <c r="H91" s="1">
@@ -11836,7 +12228,7 @@
         <v>5</v>
       </c>
       <c r="E92" s="17">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>5</v>
       </c>
     </row>
@@ -11857,7 +12249,7 @@
         <v>5</v>
       </c>
       <c r="E93" s="17">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>5</v>
       </c>
     </row>
@@ -11878,7 +12270,7 @@
         <v>5</v>
       </c>
       <c r="E94" s="17">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>5</v>
       </c>
       <c r="G94" s="33"/>
@@ -11902,7 +12294,7 @@
         <v>5</v>
       </c>
       <c r="E95" s="17">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>5</v>
       </c>
       <c r="G95" s="33"/>
@@ -11926,7 +12318,7 @@
         <v>5</v>
       </c>
       <c r="E96" s="17">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>5</v>
       </c>
       <c r="G96" s="33"/>
@@ -11950,7 +12342,7 @@
         <v>5</v>
       </c>
       <c r="E97" s="17">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>5</v>
       </c>
       <c r="G97" s="33"/>
@@ -11974,7 +12366,7 @@
         <v>5</v>
       </c>
       <c r="E98" s="17">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>5</v>
       </c>
       <c r="G98" s="33"/>
@@ -11998,7 +12390,7 @@
         <v>5</v>
       </c>
       <c r="E99" s="17">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>5</v>
       </c>
       <c r="G99" s="33"/>
@@ -12022,7 +12414,7 @@
         <v>5</v>
       </c>
       <c r="E100" s="17">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>5</v>
       </c>
     </row>
@@ -12120,7 +12512,7 @@
         <v>5</v>
       </c>
       <c r="E107" s="17">
-        <f t="shared" ref="E107:E121" si="6">AVERAGE(B107:D107)</f>
+        <f t="shared" ref="E107:E121" si="12">AVERAGE(B107:D107)</f>
         <v>5</v>
       </c>
       <c r="G107" s="34" t="s">
@@ -12148,7 +12540,7 @@
         <v>5</v>
       </c>
       <c r="E108" s="17">
-        <f t="shared" si="6"/>
+        <f t="shared" si="12"/>
         <v>5</v>
       </c>
       <c r="G108" s="34" t="s">
@@ -12176,7 +12568,7 @@
         <v>5</v>
       </c>
       <c r="E109" s="17">
-        <f t="shared" si="6"/>
+        <f t="shared" si="12"/>
         <v>5</v>
       </c>
       <c r="G109" s="34" t="s">
@@ -12204,7 +12596,7 @@
         <v>5</v>
       </c>
       <c r="E110" s="17">
-        <f t="shared" si="6"/>
+        <f t="shared" si="12"/>
         <v>5</v>
       </c>
       <c r="G110" s="34" t="s">
@@ -12232,7 +12624,7 @@
         <v>5</v>
       </c>
       <c r="E111" s="17">
-        <f t="shared" si="6"/>
+        <f t="shared" si="12"/>
         <v>5</v>
       </c>
       <c r="G111" s="34">
@@ -12260,7 +12652,7 @@
         <v>5</v>
       </c>
       <c r="E112" s="17">
-        <f t="shared" si="6"/>
+        <f t="shared" si="12"/>
         <v>5</v>
       </c>
       <c r="H112" s="1">
@@ -12285,7 +12677,7 @@
         <v>5</v>
       </c>
       <c r="E113" s="17">
-        <f t="shared" si="6"/>
+        <f t="shared" si="12"/>
         <v>5</v>
       </c>
     </row>
@@ -12306,7 +12698,7 @@
         <v>5</v>
       </c>
       <c r="E114" s="17">
-        <f t="shared" si="6"/>
+        <f t="shared" si="12"/>
         <v>5</v>
       </c>
     </row>
@@ -12327,7 +12719,7 @@
         <v>5</v>
       </c>
       <c r="E115" s="17">
-        <f t="shared" si="6"/>
+        <f t="shared" si="12"/>
         <v>5</v>
       </c>
       <c r="G115" s="33"/>
@@ -12351,7 +12743,7 @@
         <v>5</v>
       </c>
       <c r="E116" s="17">
-        <f t="shared" si="6"/>
+        <f t="shared" si="12"/>
         <v>5</v>
       </c>
       <c r="G116" s="33"/>
@@ -12375,7 +12767,7 @@
         <v>5</v>
       </c>
       <c r="E117" s="17">
-        <f t="shared" si="6"/>
+        <f t="shared" si="12"/>
         <v>5</v>
       </c>
       <c r="G117" s="33"/>
@@ -12399,7 +12791,7 @@
         <v>5</v>
       </c>
       <c r="E118" s="17">
-        <f t="shared" si="6"/>
+        <f t="shared" si="12"/>
         <v>5</v>
       </c>
       <c r="G118" s="33"/>
@@ -12423,7 +12815,7 @@
         <v>5</v>
       </c>
       <c r="E119" s="17">
-        <f t="shared" si="6"/>
+        <f t="shared" si="12"/>
         <v>5</v>
       </c>
       <c r="G119" s="33"/>
@@ -12447,7 +12839,7 @@
         <v>5</v>
       </c>
       <c r="E120" s="17">
-        <f t="shared" si="6"/>
+        <f t="shared" si="12"/>
         <v>5</v>
       </c>
       <c r="G120" s="33"/>
@@ -12471,7 +12863,7 @@
         <v>5</v>
       </c>
       <c r="E121" s="17">
-        <f t="shared" si="6"/>
+        <f t="shared" si="12"/>
         <v>5</v>
       </c>
     </row>
@@ -12569,7 +12961,7 @@
         <v>5</v>
       </c>
       <c r="E128" s="17">
-        <f t="shared" ref="E128:E142" si="7">AVERAGE(B128:D128)</f>
+        <f t="shared" ref="E128:E142" si="13">AVERAGE(B128:D128)</f>
         <v>5</v>
       </c>
       <c r="G128" s="34" t="s">
@@ -12597,7 +12989,7 @@
         <v>5</v>
       </c>
       <c r="E129" s="17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="13"/>
         <v>5</v>
       </c>
       <c r="G129" s="34" t="s">
@@ -12625,7 +13017,7 @@
         <v>5</v>
       </c>
       <c r="E130" s="17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="13"/>
         <v>5</v>
       </c>
       <c r="G130" s="34" t="s">
@@ -12653,7 +13045,7 @@
         <v>5</v>
       </c>
       <c r="E131" s="17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="13"/>
         <v>5</v>
       </c>
       <c r="G131" s="34" t="s">
@@ -12681,7 +13073,7 @@
         <v>5</v>
       </c>
       <c r="E132" s="17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="13"/>
         <v>5</v>
       </c>
       <c r="G132" s="34">
@@ -12709,7 +13101,7 @@
         <v>5</v>
       </c>
       <c r="E133" s="17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="13"/>
         <v>5</v>
       </c>
       <c r="H133" s="1">
@@ -12734,7 +13126,7 @@
         <v>5</v>
       </c>
       <c r="E134" s="17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="13"/>
         <v>5</v>
       </c>
     </row>
@@ -12755,7 +13147,7 @@
         <v>5</v>
       </c>
       <c r="E135" s="17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="13"/>
         <v>5</v>
       </c>
     </row>
@@ -12776,7 +13168,7 @@
         <v>5</v>
       </c>
       <c r="E136" s="17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="13"/>
         <v>5</v>
       </c>
       <c r="G136" s="33"/>
@@ -12799,7 +13191,7 @@
         <v>5</v>
       </c>
       <c r="E137" s="17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="13"/>
         <v>5</v>
       </c>
       <c r="G137" s="33"/>
@@ -12822,7 +13214,7 @@
         <v>5</v>
       </c>
       <c r="E138" s="17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="13"/>
         <v>5</v>
       </c>
       <c r="G138" s="33"/>
@@ -12845,7 +13237,7 @@
         <v>5</v>
       </c>
       <c r="E139" s="17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="13"/>
         <v>5</v>
       </c>
       <c r="G139" s="33"/>
@@ -12868,7 +13260,7 @@
         <v>5</v>
       </c>
       <c r="E140" s="17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="13"/>
         <v>5</v>
       </c>
       <c r="G140" s="33"/>
@@ -12891,7 +13283,7 @@
         <v>5</v>
       </c>
       <c r="E141" s="17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="13"/>
         <v>5</v>
       </c>
       <c r="G141" s="33"/>
@@ -12914,7 +13306,7 @@
         <v>5</v>
       </c>
       <c r="E142" s="17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="13"/>
         <v>5</v>
       </c>
     </row>
@@ -13012,7 +13404,7 @@
         <v>5</v>
       </c>
       <c r="E149" s="17">
-        <f t="shared" ref="E149:E163" si="8">AVERAGE(B149:D149)</f>
+        <f t="shared" ref="E149:E163" si="14">AVERAGE(B149:D149)</f>
         <v>5</v>
       </c>
       <c r="G149" s="34" t="s">
@@ -13040,7 +13432,7 @@
         <v>5</v>
       </c>
       <c r="E150" s="17">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v>5</v>
       </c>
       <c r="G150" s="34" t="s">
@@ -13068,7 +13460,7 @@
         <v>5</v>
       </c>
       <c r="E151" s="17">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v>5</v>
       </c>
       <c r="G151" s="34" t="s">
@@ -13096,7 +13488,7 @@
         <v>5</v>
       </c>
       <c r="E152" s="17">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v>5</v>
       </c>
       <c r="G152" s="34" t="s">
@@ -13124,7 +13516,7 @@
         <v>5</v>
       </c>
       <c r="E153" s="17">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v>5</v>
       </c>
       <c r="G153" s="34">
@@ -13152,7 +13544,7 @@
         <v>5</v>
       </c>
       <c r="E154" s="17">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v>5</v>
       </c>
       <c r="H154" s="1">
@@ -13177,7 +13569,7 @@
         <v>5</v>
       </c>
       <c r="E155" s="17">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v>5</v>
       </c>
     </row>
@@ -13198,7 +13590,7 @@
         <v>5</v>
       </c>
       <c r="E156" s="17">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v>5</v>
       </c>
     </row>
@@ -13219,7 +13611,7 @@
         <v>5</v>
       </c>
       <c r="E157" s="17">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v>5</v>
       </c>
       <c r="G157" s="33"/>
@@ -13243,7 +13635,7 @@
         <v>5</v>
       </c>
       <c r="E158" s="17">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v>5</v>
       </c>
       <c r="G158" s="33"/>
@@ -13267,7 +13659,7 @@
         <v>5</v>
       </c>
       <c r="E159" s="17">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v>5</v>
       </c>
       <c r="G159" s="33"/>
@@ -13291,7 +13683,7 @@
         <v>5</v>
       </c>
       <c r="E160" s="17">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v>5</v>
       </c>
       <c r="G160" s="33"/>
@@ -13315,7 +13707,7 @@
         <v>5</v>
       </c>
       <c r="E161" s="17">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v>5</v>
       </c>
       <c r="G161" s="33"/>
@@ -13339,7 +13731,7 @@
         <v>5</v>
       </c>
       <c r="E162" s="17">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v>5</v>
       </c>
       <c r="G162" s="33"/>
@@ -13363,7 +13755,7 @@
         <v>5</v>
       </c>
       <c r="E163" s="17">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v>5</v>
       </c>
     </row>
@@ -13461,7 +13853,7 @@
         <v>5</v>
       </c>
       <c r="E170" s="17">
-        <f t="shared" ref="E170:E184" si="9">AVERAGE(B170:D170)</f>
+        <f t="shared" ref="E170:E184" si="15">AVERAGE(B170:D170)</f>
         <v>5</v>
       </c>
       <c r="G170" s="34" t="s">
@@ -13489,7 +13881,7 @@
         <v>5</v>
       </c>
       <c r="E171" s="17">
-        <f t="shared" si="9"/>
+        <f t="shared" si="15"/>
         <v>5</v>
       </c>
       <c r="G171" s="34" t="s">
@@ -13517,7 +13909,7 @@
         <v>5</v>
       </c>
       <c r="E172" s="17">
-        <f t="shared" si="9"/>
+        <f t="shared" si="15"/>
         <v>5</v>
       </c>
       <c r="G172" s="34" t="s">
@@ -13545,7 +13937,7 @@
         <v>5</v>
       </c>
       <c r="E173" s="17">
-        <f t="shared" si="9"/>
+        <f t="shared" si="15"/>
         <v>5</v>
       </c>
       <c r="G173" s="34" t="s">
@@ -13573,7 +13965,7 @@
         <v>5</v>
       </c>
       <c r="E174" s="17">
-        <f t="shared" si="9"/>
+        <f t="shared" si="15"/>
         <v>5</v>
       </c>
       <c r="G174" s="34">
@@ -13601,7 +13993,7 @@
         <v>5</v>
       </c>
       <c r="E175" s="17">
-        <f t="shared" si="9"/>
+        <f t="shared" si="15"/>
         <v>5</v>
       </c>
       <c r="H175" s="1">
@@ -13626,7 +14018,7 @@
         <v>5</v>
       </c>
       <c r="E176" s="17">
-        <f t="shared" si="9"/>
+        <f t="shared" si="15"/>
         <v>5</v>
       </c>
     </row>
@@ -13647,7 +14039,7 @@
         <v>5</v>
       </c>
       <c r="E177" s="17">
-        <f t="shared" si="9"/>
+        <f t="shared" si="15"/>
         <v>5</v>
       </c>
     </row>
@@ -13668,7 +14060,7 @@
         <v>5</v>
       </c>
       <c r="E178" s="17">
-        <f t="shared" si="9"/>
+        <f t="shared" si="15"/>
         <v>5</v>
       </c>
       <c r="G178" s="33"/>
@@ -13692,7 +14084,7 @@
         <v>5</v>
       </c>
       <c r="E179" s="17">
-        <f t="shared" si="9"/>
+        <f t="shared" si="15"/>
         <v>5</v>
       </c>
       <c r="G179" s="33"/>
@@ -13716,7 +14108,7 @@
         <v>5</v>
       </c>
       <c r="E180" s="17">
-        <f t="shared" si="9"/>
+        <f t="shared" si="15"/>
         <v>5</v>
       </c>
       <c r="G180" s="33"/>
@@ -13740,7 +14132,7 @@
         <v>5</v>
       </c>
       <c r="E181" s="17">
-        <f t="shared" si="9"/>
+        <f t="shared" si="15"/>
         <v>5</v>
       </c>
       <c r="G181" s="33"/>
@@ -13764,7 +14156,7 @@
         <v>5</v>
       </c>
       <c r="E182" s="17">
-        <f t="shared" si="9"/>
+        <f t="shared" si="15"/>
         <v>5</v>
       </c>
       <c r="G182" s="33"/>
@@ -13788,7 +14180,7 @@
         <v>5</v>
       </c>
       <c r="E183" s="17">
-        <f t="shared" si="9"/>
+        <f t="shared" si="15"/>
         <v>5</v>
       </c>
       <c r="G183" s="33"/>
@@ -13812,7 +14204,7 @@
         <v>5</v>
       </c>
       <c r="E184" s="17">
-        <f t="shared" si="9"/>
+        <f t="shared" si="15"/>
         <v>5</v>
       </c>
     </row>
@@ -13910,7 +14302,7 @@
         <v>5</v>
       </c>
       <c r="E191" s="17">
-        <f t="shared" ref="E191:E205" si="10">AVERAGE(B191:D191)</f>
+        <f t="shared" ref="E191:E205" si="16">AVERAGE(B191:D191)</f>
         <v>5</v>
       </c>
       <c r="G191" s="34" t="s">
@@ -13938,7 +14330,7 @@
         <v>5</v>
       </c>
       <c r="E192" s="17">
-        <f t="shared" si="10"/>
+        <f t="shared" si="16"/>
         <v>5</v>
       </c>
       <c r="G192" s="34" t="s">
@@ -13966,7 +14358,7 @@
         <v>5</v>
       </c>
       <c r="E193" s="17">
-        <f t="shared" si="10"/>
+        <f t="shared" si="16"/>
         <v>5</v>
       </c>
       <c r="G193" s="34" t="s">
@@ -13994,7 +14386,7 @@
         <v>5</v>
       </c>
       <c r="E194" s="17">
-        <f t="shared" si="10"/>
+        <f t="shared" si="16"/>
         <v>5</v>
       </c>
       <c r="G194" s="34" t="s">
@@ -14022,7 +14414,7 @@
         <v>5</v>
       </c>
       <c r="E195" s="17">
-        <f t="shared" si="10"/>
+        <f t="shared" si="16"/>
         <v>5</v>
       </c>
       <c r="G195" s="34">
@@ -14050,7 +14442,7 @@
         <v>5</v>
       </c>
       <c r="E196" s="17">
-        <f t="shared" si="10"/>
+        <f t="shared" si="16"/>
         <v>5</v>
       </c>
       <c r="H196" s="1">
@@ -14075,7 +14467,7 @@
         <v>5</v>
       </c>
       <c r="E197" s="17">
-        <f t="shared" si="10"/>
+        <f t="shared" si="16"/>
         <v>5</v>
       </c>
     </row>
@@ -14096,7 +14488,7 @@
         <v>5</v>
       </c>
       <c r="E198" s="17">
-        <f t="shared" si="10"/>
+        <f t="shared" si="16"/>
         <v>5</v>
       </c>
     </row>
@@ -14117,7 +14509,7 @@
         <v>5</v>
       </c>
       <c r="E199" s="17">
-        <f t="shared" si="10"/>
+        <f t="shared" si="16"/>
         <v>5</v>
       </c>
       <c r="G199" s="33"/>
@@ -14141,7 +14533,7 @@
         <v>5</v>
       </c>
       <c r="E200" s="17">
-        <f t="shared" si="10"/>
+        <f t="shared" si="16"/>
         <v>5</v>
       </c>
       <c r="G200" s="33"/>
@@ -14165,7 +14557,7 @@
         <v>5</v>
       </c>
       <c r="E201" s="17">
-        <f t="shared" si="10"/>
+        <f t="shared" si="16"/>
         <v>5</v>
       </c>
       <c r="G201" s="33"/>
@@ -14189,7 +14581,7 @@
         <v>5</v>
       </c>
       <c r="E202" s="17">
-        <f t="shared" si="10"/>
+        <f t="shared" si="16"/>
         <v>5</v>
       </c>
       <c r="G202" s="33"/>
@@ -14213,7 +14605,7 @@
         <v>5</v>
       </c>
       <c r="E203" s="17">
-        <f t="shared" si="10"/>
+        <f t="shared" si="16"/>
         <v>5</v>
       </c>
       <c r="G203" s="33"/>
@@ -14237,7 +14629,7 @@
         <v>5</v>
       </c>
       <c r="E204" s="17">
-        <f t="shared" si="10"/>
+        <f t="shared" si="16"/>
         <v>5</v>
       </c>
       <c r="G204" s="33"/>
@@ -14261,7 +14653,7 @@
         <v>5</v>
       </c>
       <c r="E205" s="17">
-        <f t="shared" si="10"/>
+        <f t="shared" si="16"/>
         <v>5</v>
       </c>
     </row>
@@ -14359,7 +14751,7 @@
         <v>5</v>
       </c>
       <c r="E212" s="17">
-        <f t="shared" ref="E212:E226" si="11">AVERAGE(B212:D212)</f>
+        <f t="shared" ref="E212:E226" si="17">AVERAGE(B212:D212)</f>
         <v>5</v>
       </c>
       <c r="G212" s="34" t="s">
@@ -14387,7 +14779,7 @@
         <v>5</v>
       </c>
       <c r="E213" s="17">
-        <f t="shared" si="11"/>
+        <f t="shared" si="17"/>
         <v>5</v>
       </c>
       <c r="G213" s="34" t="s">
@@ -14415,7 +14807,7 @@
         <v>5</v>
       </c>
       <c r="E214" s="17">
-        <f t="shared" si="11"/>
+        <f t="shared" si="17"/>
         <v>5</v>
       </c>
       <c r="G214" s="34" t="s">
@@ -14443,7 +14835,7 @@
         <v>5</v>
       </c>
       <c r="E215" s="17">
-        <f t="shared" si="11"/>
+        <f t="shared" si="17"/>
         <v>5</v>
       </c>
       <c r="G215" s="34" t="s">
@@ -14471,7 +14863,7 @@
         <v>5</v>
       </c>
       <c r="E216" s="17">
-        <f t="shared" si="11"/>
+        <f t="shared" si="17"/>
         <v>5</v>
       </c>
       <c r="G216" s="34">
@@ -14499,7 +14891,7 @@
         <v>5</v>
       </c>
       <c r="E217" s="17">
-        <f t="shared" si="11"/>
+        <f t="shared" si="17"/>
         <v>5</v>
       </c>
       <c r="H217" s="1">
@@ -14524,7 +14916,7 @@
         <v>5</v>
       </c>
       <c r="E218" s="17">
-        <f t="shared" si="11"/>
+        <f t="shared" si="17"/>
         <v>5</v>
       </c>
     </row>
@@ -14545,7 +14937,7 @@
         <v>5</v>
       </c>
       <c r="E219" s="17">
-        <f t="shared" si="11"/>
+        <f t="shared" si="17"/>
         <v>5</v>
       </c>
     </row>
@@ -14566,7 +14958,7 @@
         <v>5</v>
       </c>
       <c r="E220" s="17">
-        <f t="shared" si="11"/>
+        <f t="shared" si="17"/>
         <v>5</v>
       </c>
       <c r="G220" s="33"/>
@@ -14590,7 +14982,7 @@
         <v>5</v>
       </c>
       <c r="E221" s="17">
-        <f t="shared" si="11"/>
+        <f t="shared" si="17"/>
         <v>5</v>
       </c>
       <c r="G221" s="33"/>
@@ -14614,7 +15006,7 @@
         <v>5</v>
       </c>
       <c r="E222" s="17">
-        <f t="shared" si="11"/>
+        <f t="shared" si="17"/>
         <v>5</v>
       </c>
       <c r="G222" s="33"/>
@@ -14638,7 +15030,7 @@
         <v>5</v>
       </c>
       <c r="E223" s="17">
-        <f t="shared" si="11"/>
+        <f t="shared" si="17"/>
         <v>5</v>
       </c>
       <c r="G223" s="33"/>
@@ -14662,7 +15054,7 @@
         <v>5</v>
       </c>
       <c r="E224" s="17">
-        <f t="shared" si="11"/>
+        <f t="shared" si="17"/>
         <v>5</v>
       </c>
       <c r="G224" s="33"/>
@@ -14686,7 +15078,7 @@
         <v>5</v>
       </c>
       <c r="E225" s="17">
-        <f t="shared" si="11"/>
+        <f t="shared" si="17"/>
         <v>5</v>
       </c>
       <c r="G225" s="33"/>
@@ -14710,7 +15102,7 @@
         <v>5</v>
       </c>
       <c r="E226" s="17">
-        <f t="shared" si="11"/>
+        <f t="shared" si="17"/>
         <v>5</v>
       </c>
     </row>
@@ -14808,7 +15200,7 @@
         <v>5</v>
       </c>
       <c r="E233" s="17">
-        <f t="shared" ref="E233:E247" si="12">AVERAGE(B233:D233)</f>
+        <f t="shared" ref="E233:E247" si="18">AVERAGE(B233:D233)</f>
         <v>5</v>
       </c>
       <c r="G233" s="34" t="s">
@@ -14836,7 +15228,7 @@
         <v>5</v>
       </c>
       <c r="E234" s="17">
-        <f t="shared" si="12"/>
+        <f t="shared" si="18"/>
         <v>5</v>
       </c>
       <c r="G234" s="34" t="s">
@@ -14864,7 +15256,7 @@
         <v>5</v>
       </c>
       <c r="E235" s="17">
-        <f t="shared" si="12"/>
+        <f t="shared" si="18"/>
         <v>5</v>
       </c>
       <c r="G235" s="34" t="s">
@@ -14892,7 +15284,7 @@
         <v>5</v>
       </c>
       <c r="E236" s="17">
-        <f t="shared" si="12"/>
+        <f t="shared" si="18"/>
         <v>5</v>
       </c>
       <c r="G236" s="34" t="s">
@@ -14920,7 +15312,7 @@
         <v>5</v>
       </c>
       <c r="E237" s="17">
-        <f t="shared" si="12"/>
+        <f t="shared" si="18"/>
         <v>5</v>
       </c>
       <c r="G237" s="34">
@@ -14948,7 +15340,7 @@
         <v>5</v>
       </c>
       <c r="E238" s="17">
-        <f t="shared" si="12"/>
+        <f t="shared" si="18"/>
         <v>5</v>
       </c>
       <c r="H238" s="1">
@@ -14973,7 +15365,7 @@
         <v>5</v>
       </c>
       <c r="E239" s="17">
-        <f t="shared" si="12"/>
+        <f t="shared" si="18"/>
         <v>5</v>
       </c>
     </row>
@@ -14994,7 +15386,7 @@
         <v>5</v>
       </c>
       <c r="E240" s="17">
-        <f t="shared" si="12"/>
+        <f t="shared" si="18"/>
         <v>5</v>
       </c>
     </row>
@@ -15015,7 +15407,7 @@
         <v>5</v>
       </c>
       <c r="E241" s="17">
-        <f t="shared" si="12"/>
+        <f t="shared" si="18"/>
         <v>5</v>
       </c>
       <c r="G241" s="33"/>
@@ -15039,7 +15431,7 @@
         <v>5</v>
       </c>
       <c r="E242" s="17">
-        <f t="shared" si="12"/>
+        <f t="shared" si="18"/>
         <v>5</v>
       </c>
       <c r="G242" s="33"/>
@@ -15063,7 +15455,7 @@
         <v>5</v>
       </c>
       <c r="E243" s="17">
-        <f t="shared" si="12"/>
+        <f t="shared" si="18"/>
         <v>5</v>
       </c>
       <c r="G243" s="33"/>
@@ -15087,7 +15479,7 @@
         <v>5</v>
       </c>
       <c r="E244" s="17">
-        <f t="shared" si="12"/>
+        <f t="shared" si="18"/>
         <v>5</v>
       </c>
       <c r="G244" s="33"/>
@@ -15111,7 +15503,7 @@
         <v>5</v>
       </c>
       <c r="E245" s="17">
-        <f t="shared" si="12"/>
+        <f t="shared" si="18"/>
         <v>5</v>
       </c>
       <c r="G245" s="33"/>
@@ -15135,7 +15527,7 @@
         <v>5</v>
       </c>
       <c r="E246" s="17">
-        <f t="shared" si="12"/>
+        <f t="shared" si="18"/>
         <v>5</v>
       </c>
       <c r="G246" s="33"/>
@@ -15159,7 +15551,7 @@
         <v>5</v>
       </c>
       <c r="E247" s="17">
-        <f t="shared" si="12"/>
+        <f t="shared" si="18"/>
         <v>5</v>
       </c>
     </row>

</xml_diff>